<commit_message>
Prep for next run with all countries.
</commit_message>
<xml_diff>
--- a/data/aggregation_tables/targeted_aggregations.xlsx
+++ b/data/aggregation_tables/targeted_aggregations.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkh2/github/CLPFUDecompositionDatabase/inst/aggregation_tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkh2/github/CLPFUDecompositionDatabase/data/aggregation_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB6180C2-1D4B-F94E-A664-D542D6D8044C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D5CD3D3-7531-AD4D-B592-FEABE950C36E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9920" yWindow="1680" windowWidth="17060" windowHeight="17440" activeTab="1" xr2:uid="{6196F350-644F-294F-9730-D810A8B27C87}"/>
+    <workbookView xWindow="11160" yWindow="1040" windowWidth="23420" windowHeight="14600" activeTab="2" xr2:uid="{6196F350-644F-294F-9730-D810A8B27C87}"/>
   </bookViews>
   <sheets>
     <sheet name="Meta" sheetId="2" r:id="rId1"/>
     <sheet name="industry_aggregations" sheetId="1" r:id="rId2"/>
     <sheet name="product_aggregations" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029" iterateDelta="1E-4"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="21">
   <si>
     <t>Few</t>
   </si>
@@ -69,9 +69,6 @@
     <t>across the CL-PFU database before conducting decomposition analyses.</t>
   </si>
   <si>
-    <t>ITA</t>
-  </si>
-  <si>
     <t>Coke ovens</t>
   </si>
   <si>
@@ -81,9 +78,6 @@
     <t>Gas works</t>
   </si>
   <si>
-    <t>Iron industry</t>
-  </si>
-  <si>
     <t>Renewable electricity</t>
   </si>
   <si>
@@ -103,6 +97,9 @@
   </si>
   <si>
     <t>Solar photovoltaics</t>
+  </si>
+  <si>
+    <t>Iron industry (energy)</t>
   </si>
 </sst>
 </file>
@@ -168,9 +165,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -208,7 +205,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -314,7 +311,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -456,7 +453,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -489,7 +486,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC0C3702-3414-2F44-9243-E3F7D770C663}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="20.6640625" bestFit="1" customWidth="1"/>
@@ -512,69 +509,69 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2">
-        <v>2000</v>
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3">
-        <v>2000</v>
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4">
-        <v>2001</v>
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
-        <v>2001</v>
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
         <v>10</v>
-      </c>
-      <c r="B6">
-        <v>2002</v>
-      </c>
-      <c r="C6" t="s">
-        <v>19</v>
       </c>
       <c r="D6" t="s">
         <v>20</v>
@@ -582,13 +579,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>2002</v>
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
         <v>20</v>
@@ -596,240 +593,16 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
-        <v>2003</v>
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>2003</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>2004</v>
-      </c>
-      <c r="C10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>2004</v>
-      </c>
-      <c r="C11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12">
-        <v>2005</v>
-      </c>
-      <c r="C12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13">
-        <v>2005</v>
-      </c>
-      <c r="C13" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14">
-        <v>2006</v>
-      </c>
-      <c r="C14" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15">
-        <v>2006</v>
-      </c>
-      <c r="C15" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16">
-        <v>2007</v>
-      </c>
-      <c r="C16" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17">
-        <v>2007</v>
-      </c>
-      <c r="C17" t="s">
-        <v>20</v>
-      </c>
-      <c r="D17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B18">
-        <v>2008</v>
-      </c>
-      <c r="C18" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B19">
-        <v>2008</v>
-      </c>
-      <c r="C19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D19" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B20" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>8</v>
-      </c>
-      <c r="B21" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>10</v>
-      </c>
-      <c r="B22" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>10</v>
-      </c>
-      <c r="B23" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>10</v>
-      </c>
-      <c r="B24" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -842,6 +615,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A2B3A4E-A783-2A43-8F8C-30A29FE17236}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="16.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -861,56 +637,56 @@
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2">
-        <v>2015</v>
+      <c r="B2" t="s">
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3">
-        <v>2015</v>
+      <c r="B3" t="s">
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
-        <v>2015</v>
+      <c r="B4" t="s">
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5">
-        <v>2015</v>
+      <c r="B5" t="s">
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>